<commit_message>
Full update: ColourMatch improvements, dynamic LAB scaling, backend updates
</commit_message>
<xml_diff>
--- a/src/modules/ColourMatch/data/DC Ink System.xlsx
+++ b/src/modules/ColourMatch/data/DC Ink System.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35690a85e7f049a9/Programming/PN-Pulse/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35690a85e7f049a9/ProjektNash/ProjektNash-Core/src/modules/ColourMatch/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F25DC773A252ABDACC104871795E4A045BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE9A42CE-5D42-49F8-97C9-1541BA0CA03D}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="11_F25DC773A252ABDACC104871795E4A045BDE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC60FB0C-E009-4460-8D87-4D7C54B35DAF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="29">
   <si>
     <t>Ink</t>
   </si>
@@ -76,6 +76,42 @@
   </si>
   <si>
     <t>DC21-802</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Extender</t>
+  </si>
+  <si>
+    <t>HR Violet</t>
+  </si>
+  <si>
+    <t>Royal Blue</t>
+  </si>
+  <si>
+    <t>Process Blue</t>
+  </si>
+  <si>
+    <t>Mixing Black</t>
+  </si>
+  <si>
+    <t>HR Bright Red</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warm Red</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rhodamine</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Orange</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yellow</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Green</t>
   </si>
 </sst>
 </file>
@@ -136,7 +172,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -422,1762 +458,2070 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="9.28515625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="2" max="2" width="22" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="9.28515625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2" s="1">
         <v>94.9</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>1.2</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>-3.4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1">
         <v>100</v>
       </c>
-      <c r="C3" s="1">
+      <c r="D3" s="1">
         <v>93.4</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>-0.6</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>0.7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="1">
         <v>0.5</v>
       </c>
-      <c r="C4" s="1">
+      <c r="D4" s="1">
         <v>91.7</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>2.4</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="1">
+      <c r="D5" s="1">
         <v>90</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>5</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>0.7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="1">
+      <c r="D6" s="1">
         <v>87.4</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>9.3000000000000007</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>1.7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="1">
         <v>4</v>
       </c>
-      <c r="C7" s="1">
+      <c r="D7" s="1">
         <v>83.2</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>16.399999999999999</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>1.8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="1">
         <v>8</v>
       </c>
-      <c r="C8" s="1">
+      <c r="D8" s="1">
         <v>76.7</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>27.2</v>
       </c>
-      <c r="E8" s="1">
+      <c r="F8" s="1">
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="1">
         <v>16</v>
       </c>
-      <c r="C9" s="1">
+      <c r="D9" s="1">
         <v>68.7</v>
       </c>
-      <c r="D9" s="1">
+      <c r="E9" s="1">
         <v>41.1</v>
       </c>
-      <c r="E9" s="1">
+      <c r="F9" s="1">
         <v>8.6</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1">
         <v>32</v>
       </c>
-      <c r="C10" s="1">
+      <c r="D10" s="1">
         <v>59.9</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>56.7</v>
       </c>
-      <c r="E10" s="1">
+      <c r="F10" s="1">
         <v>16.8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="1">
         <v>64</v>
       </c>
-      <c r="C11" s="1">
+      <c r="D11" s="1">
         <v>51</v>
       </c>
-      <c r="D11" s="1">
+      <c r="E11" s="1">
         <v>71.5</v>
       </c>
-      <c r="E11" s="1">
+      <c r="F11" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="1">
         <v>80</v>
       </c>
-      <c r="C12" s="1">
+      <c r="D12" s="1">
         <v>48.9</v>
       </c>
-      <c r="D12" s="1">
+      <c r="E12" s="1">
         <v>74</v>
       </c>
-      <c r="E12" s="1">
+      <c r="F12" s="1">
         <v>43.6</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="1">
         <v>100</v>
       </c>
-      <c r="C13" s="1">
+      <c r="D13" s="1">
         <v>47.4</v>
       </c>
-      <c r="D13" s="1">
+      <c r="E13" s="1">
         <v>75</v>
       </c>
-      <c r="E13" s="1">
+      <c r="F13" s="1">
         <v>51.4</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1">
         <v>0.5</v>
       </c>
-      <c r="C14" s="1">
+      <c r="D14" s="1">
         <v>91</v>
       </c>
-      <c r="D14" s="1">
+      <c r="E14" s="1">
         <v>5.3</v>
       </c>
-      <c r="E14" s="1">
+      <c r="F14" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="1">
         <v>1</v>
       </c>
-      <c r="C15" s="1">
+      <c r="D15" s="1">
         <v>89.2</v>
       </c>
-      <c r="D15" s="1">
+      <c r="E15" s="1">
         <v>9.8000000000000007</v>
       </c>
-      <c r="E15" s="1">
+      <c r="F15" s="1">
         <v>-0.5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="1">
         <v>2</v>
       </c>
-      <c r="C16" s="1">
+      <c r="D16" s="1">
         <v>86.4</v>
       </c>
-      <c r="D16" s="1">
+      <c r="E16" s="1">
         <v>16.5</v>
       </c>
-      <c r="E16" s="1">
+      <c r="F16" s="1">
         <v>-0.7</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="1">
         <v>4</v>
       </c>
-      <c r="C17" s="1">
+      <c r="D17" s="1">
         <v>82.1</v>
       </c>
-      <c r="D17" s="1">
+      <c r="E17" s="1">
         <v>26.5</v>
       </c>
-      <c r="E17" s="1">
+      <c r="F17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="1">
         <v>8</v>
       </c>
-      <c r="C18" s="1">
+      <c r="D18" s="1">
         <v>76.400000000000006</v>
       </c>
-      <c r="D18" s="1">
+      <c r="E18" s="1">
         <v>38.6</v>
       </c>
-      <c r="E18" s="1">
+      <c r="F18" s="1">
         <v>2.7</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="1">
         <v>16</v>
       </c>
-      <c r="C19" s="1">
+      <c r="D19" s="1">
         <v>69.900000000000006</v>
       </c>
-      <c r="D19" s="1">
+      <c r="E19" s="1">
         <v>51.7</v>
       </c>
-      <c r="E19" s="1">
+      <c r="F19" s="1">
         <v>8.6</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="1">
         <v>32</v>
       </c>
-      <c r="C20" s="1">
+      <c r="D20" s="1">
         <v>63.9</v>
       </c>
-      <c r="D20" s="1">
+      <c r="E20" s="1">
         <v>62.6</v>
       </c>
-      <c r="E20" s="1">
+      <c r="F20" s="1">
         <v>18.2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="1">
         <v>64</v>
       </c>
-      <c r="C21" s="1">
+      <c r="D21" s="1">
         <v>57.2</v>
       </c>
-      <c r="D21" s="1">
+      <c r="E21" s="1">
         <v>69.8</v>
       </c>
-      <c r="E21" s="1">
+      <c r="F21" s="1">
         <v>41.3</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="1">
         <v>80</v>
       </c>
-      <c r="C22" s="1">
+      <c r="D22" s="1">
         <v>55.9</v>
       </c>
-      <c r="D22" s="1">
+      <c r="E22" s="1">
         <v>70.599999999999994</v>
       </c>
-      <c r="E22" s="1">
+      <c r="F22" s="1">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="1">
         <v>100</v>
       </c>
-      <c r="C23" s="1">
+      <c r="D23" s="1">
         <v>54.2</v>
       </c>
-      <c r="D23" s="1">
+      <c r="E23" s="1">
         <v>71.099999999999994</v>
       </c>
-      <c r="E23" s="1">
+      <c r="F23" s="1">
         <v>59.3</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="1">
         <v>0.5</v>
       </c>
-      <c r="C24" s="1">
+      <c r="D24" s="1">
         <v>91.7</v>
       </c>
-      <c r="D24" s="1">
+      <c r="E24" s="1">
         <v>2.5</v>
       </c>
-      <c r="E24" s="1">
+      <c r="F24" s="1">
         <v>-0.8</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="1">
         <v>1</v>
       </c>
-      <c r="C25" s="1">
+      <c r="D25" s="1">
         <v>90.4</v>
       </c>
-      <c r="D25" s="1">
+      <c r="E25" s="1">
         <v>5.4</v>
       </c>
-      <c r="E25" s="1">
+      <c r="F25" s="1">
         <v>-2.5</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="1">
         <v>2</v>
       </c>
-      <c r="C26" s="1">
+      <c r="D26" s="1">
         <v>88.1</v>
       </c>
-      <c r="D26" s="1">
+      <c r="E26" s="1">
         <v>10.1</v>
       </c>
-      <c r="E26" s="1">
+      <c r="F26" s="1">
         <v>-4.8</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="1">
         <v>4</v>
       </c>
-      <c r="C27" s="1">
+      <c r="D27" s="1">
         <v>83.9</v>
       </c>
-      <c r="D27" s="1">
+      <c r="E27" s="1">
         <v>18.399999999999999</v>
       </c>
-      <c r="E27" s="1">
+      <c r="F27" s="1">
         <v>-8.8000000000000007</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="1">
         <v>8</v>
       </c>
-      <c r="C28" s="1">
+      <c r="D28" s="1">
         <v>78.7</v>
       </c>
-      <c r="D28" s="1">
+      <c r="E28" s="1">
         <v>28.5</v>
       </c>
-      <c r="E28" s="1">
+      <c r="F28" s="1">
         <v>-13.2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="1">
         <v>16</v>
       </c>
-      <c r="C29" s="1">
+      <c r="D29" s="1">
         <v>71.900000000000006</v>
       </c>
-      <c r="D29" s="1">
+      <c r="E29" s="1">
         <v>41.8</v>
       </c>
-      <c r="E29" s="1">
+      <c r="F29" s="1">
         <v>-17.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="1">
         <v>32</v>
       </c>
-      <c r="C30" s="1">
+      <c r="D30" s="1">
         <v>61.8</v>
       </c>
-      <c r="D30" s="1">
+      <c r="E30" s="1">
         <v>58.7</v>
       </c>
-      <c r="E30" s="1">
+      <c r="F30" s="1">
         <v>-21.4</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="1">
         <v>64</v>
       </c>
-      <c r="C31" s="1">
+      <c r="D31" s="1">
         <v>52.5</v>
       </c>
-      <c r="D31" s="1">
+      <c r="E31" s="1">
         <v>72.2</v>
       </c>
-      <c r="E31" s="1">
+      <c r="F31" s="1">
         <v>-22.4</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="1">
         <v>80</v>
       </c>
-      <c r="C32" s="1">
+      <c r="D32" s="1">
         <v>49.4</v>
       </c>
-      <c r="D32" s="1">
+      <c r="E32" s="1">
         <v>75.5</v>
       </c>
-      <c r="E32" s="1">
+      <c r="F32" s="1">
         <v>-21</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" s="1">
         <v>100</v>
       </c>
-      <c r="C33" s="1">
+      <c r="D33" s="1">
         <v>47.2</v>
       </c>
-      <c r="D33" s="1">
+      <c r="E33" s="1">
         <v>77.2</v>
       </c>
-      <c r="E33" s="1">
+      <c r="F33" s="1">
         <v>-20.8</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="1">
         <v>0.5</v>
       </c>
-      <c r="C34" s="1">
+      <c r="D34" s="1">
         <v>92.1</v>
       </c>
-      <c r="D34" s="1">
+      <c r="E34" s="1">
         <v>1.3</v>
       </c>
-      <c r="E34" s="1">
+      <c r="F34" s="1">
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="1">
         <v>1</v>
       </c>
-      <c r="C35" s="1">
+      <c r="D35" s="1">
         <v>91.1</v>
       </c>
-      <c r="D35" s="1">
+      <c r="E35" s="1">
         <v>3</v>
       </c>
-      <c r="E35" s="1">
+      <c r="F35" s="1">
         <v>7.5</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="1">
         <v>2</v>
       </c>
-      <c r="C36" s="1">
+      <c r="D36" s="1">
         <v>89.3</v>
       </c>
-      <c r="D36" s="1">
+      <c r="E36" s="1">
         <v>5.8</v>
       </c>
-      <c r="E36" s="1">
+      <c r="F36" s="1">
         <v>12.5</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" s="1">
         <v>4</v>
       </c>
-      <c r="C37" s="1">
+      <c r="D37" s="1">
         <v>86.8</v>
       </c>
-      <c r="D37" s="1">
+      <c r="E37" s="1">
         <v>10.4</v>
       </c>
-      <c r="E37" s="1">
+      <c r="F37" s="1">
         <v>19.899999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" s="1">
         <v>8</v>
       </c>
-      <c r="C38" s="1">
+      <c r="D38" s="1">
         <v>82.9</v>
       </c>
-      <c r="D38" s="1">
+      <c r="E38" s="1">
         <v>17.5</v>
       </c>
-      <c r="E38" s="1">
+      <c r="F38" s="1">
         <v>31.1</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C39" s="1">
         <v>16</v>
       </c>
-      <c r="C39" s="1">
+      <c r="D39" s="1">
         <v>78.400000000000006</v>
       </c>
-      <c r="D39" s="1">
+      <c r="E39" s="1">
         <v>26.2</v>
       </c>
-      <c r="E39" s="1">
+      <c r="F39" s="1">
         <v>45.7</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" s="1">
         <v>32</v>
       </c>
-      <c r="C40" s="1">
+      <c r="D40" s="1">
         <v>73</v>
       </c>
-      <c r="D40" s="1">
+      <c r="E40" s="1">
         <v>37.200000000000003</v>
       </c>
-      <c r="E40" s="1">
+      <c r="F40" s="1">
         <v>66.599999999999994</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C41" s="1">
         <v>64</v>
       </c>
-      <c r="C41" s="1">
+      <c r="D41" s="1">
         <v>67.900000000000006</v>
       </c>
-      <c r="D41" s="1">
+      <c r="E41" s="1">
         <v>47.8</v>
       </c>
-      <c r="E41" s="1">
+      <c r="F41" s="1">
         <v>88.3</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C42" s="1">
         <v>80</v>
       </c>
-      <c r="C42" s="1">
+      <c r="D42" s="1">
         <v>66.3</v>
       </c>
-      <c r="D42" s="1">
+      <c r="E42" s="1">
         <v>51.2</v>
       </c>
-      <c r="E42" s="1">
+      <c r="F42" s="1">
         <v>94.6</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" s="1">
         <v>100</v>
       </c>
-      <c r="C43" s="1">
+      <c r="D43" s="1">
         <v>65.2</v>
       </c>
-      <c r="D43" s="1">
+      <c r="E43" s="1">
         <v>52.4</v>
       </c>
-      <c r="E43" s="1">
+      <c r="F43" s="1">
         <v>95.2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C44" s="1">
         <v>0.5</v>
       </c>
-      <c r="C44" s="1">
+      <c r="D44" s="1">
         <v>93.1</v>
       </c>
-      <c r="D44" s="1">
+      <c r="E44" s="1">
         <v>-2</v>
       </c>
-      <c r="E44" s="1">
+      <c r="F44" s="1">
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="1">
         <v>1</v>
       </c>
-      <c r="C45" s="1">
+      <c r="D45" s="1">
         <v>93</v>
       </c>
-      <c r="D45" s="1">
+      <c r="E45" s="1">
         <v>-3</v>
       </c>
-      <c r="E45" s="1">
+      <c r="F45" s="1">
         <v>8.3000000000000007</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" s="1">
         <v>2</v>
       </c>
-      <c r="C46" s="1">
+      <c r="D46" s="1">
         <v>92.8</v>
       </c>
-      <c r="D46" s="1">
+      <c r="E46" s="1">
         <v>-4.5999999999999996</v>
       </c>
-      <c r="E46" s="1">
+      <c r="F46" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47" s="1">
         <v>4</v>
       </c>
-      <c r="C47" s="1">
+      <c r="D47" s="1">
         <v>92.3</v>
       </c>
-      <c r="D47" s="1">
+      <c r="E47" s="1">
         <v>-7.1</v>
       </c>
-      <c r="E47" s="1">
+      <c r="F47" s="1">
         <v>24.2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C48" s="1">
         <v>8</v>
       </c>
-      <c r="C48" s="1">
+      <c r="D48" s="1">
         <v>91.7</v>
       </c>
-      <c r="D48" s="1">
+      <c r="E48" s="1">
         <v>-9.8000000000000007</v>
       </c>
-      <c r="E48" s="1">
+      <c r="F48" s="1">
         <v>37.9</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="1">
         <v>16</v>
       </c>
-      <c r="C49" s="1">
+      <c r="D49" s="1">
         <v>91</v>
       </c>
-      <c r="D49" s="1">
+      <c r="E49" s="1">
         <v>-11.9</v>
       </c>
-      <c r="E49" s="1">
+      <c r="F49" s="1">
         <v>55.4</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50" s="1">
         <v>32</v>
       </c>
-      <c r="C50" s="1">
+      <c r="D50" s="1">
         <v>90</v>
       </c>
-      <c r="D50" s="1">
+      <c r="E50" s="1">
         <v>-13.1</v>
       </c>
-      <c r="E50" s="1">
+      <c r="F50" s="1">
         <v>80.099999999999994</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B51" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51" s="1">
         <v>64</v>
       </c>
-      <c r="C51" s="1">
+      <c r="D51" s="1">
         <v>89.3</v>
       </c>
-      <c r="D51" s="1">
+      <c r="E51" s="1">
         <v>-11.6</v>
       </c>
-      <c r="E51" s="1">
+      <c r="F51" s="1">
         <v>98.3</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B52" s="1">
+      <c r="B52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C52" s="1">
         <v>80</v>
       </c>
-      <c r="C52" s="1">
+      <c r="D52" s="1">
         <v>88.6</v>
       </c>
-      <c r="D52" s="1">
+      <c r="E52" s="1">
         <v>-10.7</v>
       </c>
-      <c r="E52" s="1">
+      <c r="F52" s="1">
         <v>110.3</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C53" s="1">
         <v>100</v>
       </c>
-      <c r="C53" s="1">
+      <c r="D53" s="1">
         <v>88</v>
       </c>
-      <c r="D53" s="1">
+      <c r="E53" s="1">
         <v>-9.9</v>
       </c>
-      <c r="E53" s="1">
+      <c r="F53" s="1">
         <v>112.2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C54" s="1">
         <v>0.5</v>
       </c>
-      <c r="C54" s="1">
+      <c r="D54" s="1">
         <v>92.5</v>
       </c>
-      <c r="D54" s="1">
+      <c r="E54" s="1">
         <v>-4</v>
       </c>
-      <c r="E54" s="1">
+      <c r="F54" s="1">
         <v>0.1</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="1">
+      <c r="B55" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55" s="1">
         <v>1</v>
       </c>
-      <c r="C55" s="1">
+      <c r="D55" s="1">
         <v>91.4</v>
       </c>
-      <c r="D55" s="1">
+      <c r="E55" s="1">
         <v>-6.8</v>
       </c>
-      <c r="E55" s="1">
+      <c r="F55" s="1">
         <v>-0.6</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B56" s="1">
+      <c r="B56" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" s="1">
         <v>2</v>
       </c>
-      <c r="C56" s="1">
+      <c r="D56" s="1">
         <v>90</v>
       </c>
-      <c r="D56" s="1">
+      <c r="E56" s="1">
         <v>-11.7</v>
       </c>
-      <c r="E56" s="1">
+      <c r="F56" s="1">
         <v>-1.1000000000000001</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B57" s="1">
+      <c r="B57" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" s="1">
         <v>4</v>
       </c>
-      <c r="C57" s="1">
+      <c r="D57" s="1">
         <v>87.5</v>
       </c>
-      <c r="D57" s="1">
+      <c r="E57" s="1">
         <v>-18.600000000000001</v>
       </c>
-      <c r="E57" s="1">
+      <c r="F57" s="1">
         <v>-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="1">
+      <c r="B58" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C58" s="1">
         <v>8</v>
       </c>
-      <c r="C58" s="1">
+      <c r="D58" s="1">
         <v>83.7</v>
       </c>
-      <c r="D58" s="1">
+      <c r="E58" s="1">
         <v>-29.2</v>
       </c>
-      <c r="E58" s="1">
+      <c r="F58" s="1">
         <v>-2.2000000000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B59" s="1">
+      <c r="B59" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C59" s="1">
         <v>16</v>
       </c>
-      <c r="C59" s="1">
+      <c r="D59" s="1">
         <v>78.900000000000006</v>
       </c>
-      <c r="D59" s="1">
+      <c r="E59" s="1">
         <v>-41.1</v>
       </c>
-      <c r="E59" s="1">
+      <c r="F59" s="1">
         <v>-1.9</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B60" s="1">
+      <c r="B60" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" s="1">
         <v>32</v>
       </c>
-      <c r="C60" s="1">
+      <c r="D60" s="1">
         <v>71.5</v>
       </c>
-      <c r="D60" s="1">
+      <c r="E60" s="1">
         <v>-57.1</v>
       </c>
-      <c r="E60" s="1">
+      <c r="F60" s="1">
         <v>-0.7</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B61" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" s="1">
         <v>64</v>
       </c>
-      <c r="C61" s="1">
+      <c r="D61" s="1">
         <v>62.9</v>
       </c>
-      <c r="D61" s="1">
+      <c r="E61" s="1">
         <v>-71.900000000000006</v>
       </c>
-      <c r="E61" s="1">
+      <c r="F61" s="1">
         <v>1.9</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="1">
+      <c r="B62" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62" s="1">
         <v>80</v>
       </c>
-      <c r="C62" s="1">
+      <c r="D62" s="1">
         <v>59.5</v>
       </c>
-      <c r="D62" s="1">
+      <c r="E62" s="1">
         <v>-76.400000000000006</v>
       </c>
-      <c r="E62" s="1">
+      <c r="F62" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="1">
+      <c r="B63" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" s="1">
         <v>100</v>
       </c>
-      <c r="C63" s="1">
+      <c r="D63" s="1">
         <v>56</v>
       </c>
-      <c r="D63" s="1">
+      <c r="E63" s="1">
         <v>-80.099999999999994</v>
       </c>
-      <c r="E63" s="1">
+      <c r="F63" s="1">
         <v>4.3</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B64" s="1">
+      <c r="B64" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C64" s="1">
         <v>0.5</v>
       </c>
-      <c r="C64" s="1">
+      <c r="D64" s="1">
         <v>91.1</v>
       </c>
-      <c r="D64" s="1">
+      <c r="E64" s="1">
         <v>-4.5999999999999996</v>
       </c>
-      <c r="E64" s="1">
+      <c r="F64" s="1">
         <v>-2.7</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B65" s="1">
+      <c r="B65" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="1">
         <v>1</v>
       </c>
-      <c r="C65" s="1">
+      <c r="D65" s="1">
         <v>89.2</v>
       </c>
-      <c r="D65" s="1">
+      <c r="E65" s="1">
         <v>-4.5999999999999996</v>
       </c>
-      <c r="E65" s="1">
+      <c r="F65" s="1">
         <v>-5.5</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B66" s="1">
+      <c r="B66" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C66" s="1">
         <v>2</v>
       </c>
-      <c r="C66" s="1">
+      <c r="D66" s="1">
         <v>86.1</v>
       </c>
-      <c r="D66" s="1">
+      <c r="E66" s="1">
         <v>-7.7</v>
       </c>
-      <c r="E66" s="1">
+      <c r="F66" s="1">
         <v>-10.6</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B67" s="1">
+      <c r="B67" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C67" s="1">
         <v>4</v>
       </c>
-      <c r="C67" s="1">
+      <c r="D67" s="1">
         <v>81.599999999999994</v>
       </c>
-      <c r="D67" s="1">
+      <c r="E67" s="1">
         <v>-11.8</v>
       </c>
-      <c r="E67" s="1">
+      <c r="F67" s="1">
         <v>-17.3</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="1">
+      <c r="B68" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" s="1">
         <v>8</v>
       </c>
-      <c r="C68" s="1">
+      <c r="D68" s="1">
         <v>75.900000000000006</v>
       </c>
-      <c r="D68" s="1">
+      <c r="E68" s="1">
         <v>-17</v>
       </c>
-      <c r="E68" s="1">
+      <c r="F68" s="1">
         <v>-25.3</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B69" s="1">
+      <c r="B69" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C69" s="1">
         <v>16</v>
       </c>
-      <c r="C69" s="1">
+      <c r="D69" s="1">
         <v>68.099999999999994</v>
       </c>
-      <c r="D69" s="1">
+      <c r="E69" s="1">
         <v>-22</v>
       </c>
-      <c r="E69" s="1">
+      <c r="F69" s="1">
         <v>-35.299999999999997</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B70" s="1">
+      <c r="B70" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C70" s="1">
         <v>32</v>
       </c>
-      <c r="C70" s="1">
+      <c r="D70" s="1">
         <v>58.3</v>
       </c>
-      <c r="D70" s="1">
+      <c r="E70" s="1">
         <v>-26.8</v>
       </c>
-      <c r="E70" s="1">
+      <c r="F70" s="1">
         <v>-46.3</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B71" s="1">
+      <c r="B71" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C71" s="1">
         <v>64</v>
       </c>
-      <c r="C71" s="1">
+      <c r="D71" s="1">
         <v>49</v>
       </c>
-      <c r="D71" s="1">
+      <c r="E71" s="1">
         <v>-28.2</v>
       </c>
-      <c r="E71" s="1">
+      <c r="F71" s="1">
         <v>-54</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B72" s="1">
+      <c r="B72" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C72" s="1">
         <v>80</v>
       </c>
-      <c r="C72" s="1">
+      <c r="D72" s="1">
         <v>45.3</v>
       </c>
-      <c r="D72" s="1">
+      <c r="E72" s="1">
         <v>-21.9</v>
       </c>
-      <c r="E72" s="1">
+      <c r="F72" s="1">
         <v>-56</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B73" s="1">
+      <c r="B73" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C73" s="1">
         <v>100</v>
       </c>
-      <c r="C73" s="1">
+      <c r="D73" s="1">
         <v>42</v>
       </c>
-      <c r="D73" s="1">
+      <c r="E73" s="1">
         <v>-17.3</v>
       </c>
-      <c r="E73" s="1">
+      <c r="F73" s="1">
         <v>-57.2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B74" s="1">
+      <c r="B74" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C74" s="1">
         <v>0.5</v>
       </c>
-      <c r="C74" s="1">
+      <c r="D74" s="1">
         <v>89.8</v>
       </c>
-      <c r="D74" s="1">
+      <c r="E74" s="1">
         <v>-0.2</v>
       </c>
-      <c r="E74" s="1">
+      <c r="F74" s="1">
         <v>-4</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B75" s="1">
+      <c r="B75" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C75" s="1">
         <v>1</v>
       </c>
-      <c r="C75" s="1">
+      <c r="D75" s="1">
         <v>86.6</v>
       </c>
-      <c r="D75" s="1">
+      <c r="E75" s="1">
         <v>0.5</v>
       </c>
-      <c r="E75" s="1">
+      <c r="F75" s="1">
         <v>-8.5</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B76" s="1">
+      <c r="B76" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C76" s="1">
         <v>2</v>
       </c>
-      <c r="C76" s="1">
+      <c r="D76" s="1">
         <v>82.1</v>
       </c>
-      <c r="D76" s="1">
+      <c r="E76" s="1">
         <v>1.9</v>
       </c>
-      <c r="E76" s="1">
+      <c r="F76" s="1">
         <v>-15.2</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B77" s="1">
+      <c r="B77" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C77" s="1">
         <v>4</v>
       </c>
-      <c r="C77" s="1">
+      <c r="D77" s="1">
         <v>75.400000000000006</v>
       </c>
-      <c r="D77" s="1">
+      <c r="E77" s="1">
         <v>4</v>
       </c>
-      <c r="E77" s="1">
+      <c r="F77" s="1">
         <v>-23.2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B78" s="1">
+      <c r="B78" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C78" s="1">
         <v>8</v>
       </c>
-      <c r="C78" s="1">
+      <c r="D78" s="1">
         <v>65.5</v>
       </c>
-      <c r="D78" s="1">
+      <c r="E78" s="1">
         <v>8.6999999999999993</v>
       </c>
-      <c r="E78" s="1">
+      <c r="F78" s="1">
         <v>-34.9</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B79" s="1">
+      <c r="B79" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C79" s="1">
         <v>16</v>
       </c>
-      <c r="C79" s="1">
+      <c r="D79" s="1">
         <v>53.3</v>
       </c>
-      <c r="D79" s="1">
+      <c r="E79" s="1">
         <v>15.8</v>
       </c>
-      <c r="E79" s="1">
+      <c r="F79" s="1">
         <v>-47.9</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B80" s="1">
+      <c r="B80" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C80" s="1">
         <v>32</v>
       </c>
-      <c r="C80" s="1">
+      <c r="D80" s="1">
         <v>37.4</v>
       </c>
-      <c r="D80" s="1">
+      <c r="E80" s="1">
         <v>28.6</v>
       </c>
-      <c r="E80" s="1">
+      <c r="F80" s="1">
         <v>-61.7</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B81" s="1">
+      <c r="B81" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C81" s="1">
         <v>64</v>
       </c>
-      <c r="C81" s="1">
+      <c r="D81" s="1">
         <v>23</v>
       </c>
-      <c r="D81" s="1">
+      <c r="E81" s="1">
         <v>45</v>
       </c>
-      <c r="E81" s="1">
+      <c r="F81" s="1">
         <v>-70.099999999999994</v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B82" s="1">
+      <c r="B82" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C82" s="1">
         <v>80</v>
       </c>
-      <c r="C82" s="1">
+      <c r="D82" s="1">
         <v>18.600000000000001</v>
       </c>
-      <c r="D82" s="1">
+      <c r="E82" s="1">
         <v>49.1</v>
       </c>
-      <c r="E82" s="1">
+      <c r="F82" s="1">
         <v>-69.8</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B83" s="1">
+      <c r="B83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="1">
         <v>100</v>
       </c>
-      <c r="C83" s="1">
+      <c r="D83" s="1">
         <v>16.3</v>
       </c>
-      <c r="D83" s="1">
+      <c r="E83" s="1">
         <v>51.4</v>
       </c>
-      <c r="E83" s="1">
+      <c r="F83" s="1">
         <v>-69.400000000000006</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B84" s="1">
+      <c r="B84" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C84" s="1">
         <v>0.5</v>
       </c>
-      <c r="C84" s="1">
+      <c r="D84" s="1">
         <v>90.5</v>
       </c>
-      <c r="D84" s="1">
+      <c r="E84" s="1">
         <v>2.8</v>
       </c>
-      <c r="E84" s="1">
+      <c r="F84" s="1">
         <v>-3.1</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B85" s="1">
+      <c r="B85" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85" s="1">
         <v>1</v>
       </c>
-      <c r="C85" s="1">
+      <c r="D85" s="1">
         <v>87.9</v>
       </c>
-      <c r="D85" s="1">
+      <c r="E85" s="1">
         <v>5.8</v>
       </c>
-      <c r="E85" s="1">
+      <c r="F85" s="1">
         <v>-6.7</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B86" s="1">
+      <c r="B86" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C86" s="1">
         <v>2</v>
       </c>
-      <c r="C86" s="1">
+      <c r="D86" s="1">
         <v>83.3</v>
       </c>
-      <c r="D86" s="1">
+      <c r="E86" s="1">
         <v>10.3</v>
       </c>
-      <c r="E86" s="1">
+      <c r="F86" s="1">
         <v>-12.2</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B87" s="1">
+      <c r="B87" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C87" s="1">
         <v>4</v>
       </c>
-      <c r="C87" s="1">
+      <c r="D87" s="1">
         <v>76.8</v>
       </c>
-      <c r="D87" s="1">
+      <c r="E87" s="1">
         <v>17</v>
       </c>
-      <c r="E87" s="1">
+      <c r="F87" s="1">
         <v>-20.399999999999999</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B88" s="1">
+      <c r="B88" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C88" s="1">
         <v>8</v>
       </c>
-      <c r="C88" s="1">
+      <c r="D88" s="1">
         <v>67.900000000000006</v>
       </c>
-      <c r="D88" s="1">
+      <c r="E88" s="1">
         <v>25.1</v>
       </c>
-      <c r="E88" s="1">
+      <c r="F88" s="1">
         <v>-30.2</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B89" s="1">
+      <c r="B89" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C89" s="1">
         <v>16</v>
       </c>
-      <c r="C89" s="1">
+      <c r="D89" s="1">
         <v>55.1</v>
       </c>
-      <c r="D89" s="1">
+      <c r="E89" s="1">
         <v>36.5</v>
       </c>
-      <c r="E89" s="1">
+      <c r="F89" s="1">
         <v>-42.2</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B90" s="1">
+      <c r="B90" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C90" s="1">
         <v>32</v>
       </c>
-      <c r="C90" s="1">
+      <c r="D90" s="1">
         <v>41.7</v>
       </c>
-      <c r="D90" s="1">
+      <c r="E90" s="1">
         <v>48.4</v>
       </c>
-      <c r="E90" s="1">
+      <c r="F90" s="1">
         <v>-53.4</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B91" s="1">
+      <c r="B91" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C91" s="1">
         <v>64</v>
       </c>
-      <c r="C91" s="1">
+      <c r="D91" s="1">
         <v>26.2</v>
       </c>
-      <c r="D91" s="1">
+      <c r="E91" s="1">
         <v>59.8</v>
       </c>
-      <c r="E91" s="1">
+      <c r="F91" s="1">
         <v>-62.1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B92" s="1">
+      <c r="B92" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C92" s="1">
         <v>80</v>
       </c>
-      <c r="C92" s="1">
+      <c r="D92" s="1">
         <v>20.100000000000001</v>
       </c>
-      <c r="D92" s="1">
+      <c r="E92" s="1">
         <v>61.4</v>
       </c>
-      <c r="E92" s="1">
+      <c r="F92" s="1">
         <v>-62.7</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B93" s="1">
+      <c r="B93" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C93" s="1">
         <v>100</v>
       </c>
-      <c r="C93" s="1">
+      <c r="D93" s="1">
         <v>18.100000000000001</v>
       </c>
-      <c r="D93" s="1">
+      <c r="E93" s="1">
         <v>61.4</v>
       </c>
-      <c r="E93" s="1">
+      <c r="F93" s="1">
         <v>-62.5</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B94" s="1">
+      <c r="B94" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C94" s="1">
         <v>0.5</v>
       </c>
-      <c r="C94" s="1">
+      <c r="D94" s="1">
         <v>90.2</v>
       </c>
-      <c r="D94" s="1">
+      <c r="E94" s="1">
         <v>-0.4</v>
       </c>
-      <c r="E94" s="1">
+      <c r="F94" s="1">
         <v>1.6</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B95" s="1">
+      <c r="B95" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C95" s="1">
         <v>1</v>
       </c>
-      <c r="C95" s="1">
+      <c r="D95" s="1">
         <v>87.6</v>
       </c>
-      <c r="D95" s="1">
+      <c r="E95" s="1">
         <v>-0.2</v>
       </c>
-      <c r="E95" s="1">
+      <c r="F95" s="1">
         <v>1.8</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B96" s="1">
+      <c r="B96" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C96" s="1">
         <v>2</v>
       </c>
-      <c r="C96" s="1">
+      <c r="D96" s="1">
         <v>83</v>
       </c>
-      <c r="D96" s="1">
+      <c r="E96" s="1">
         <v>0</v>
       </c>
-      <c r="E96" s="1">
+      <c r="F96" s="1">
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B97" s="1">
+      <c r="B97" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C97" s="1">
         <v>4</v>
       </c>
-      <c r="C97" s="1">
+      <c r="D97" s="1">
         <v>76.3</v>
       </c>
-      <c r="D97" s="1">
+      <c r="E97" s="1">
         <v>0.3</v>
       </c>
-      <c r="E97" s="1">
+      <c r="F97" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B98" s="1">
+      <c r="B98" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C98" s="1">
         <v>8</v>
       </c>
-      <c r="C98" s="1">
+      <c r="D98" s="1">
         <v>65.099999999999994</v>
       </c>
-      <c r="D98" s="1">
+      <c r="E98" s="1">
         <v>0.6</v>
       </c>
-      <c r="E98" s="1">
+      <c r="F98" s="1">
         <v>4.2</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B99" s="1">
+      <c r="B99" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C99" s="1">
         <v>16</v>
       </c>
-      <c r="C99" s="1">
+      <c r="D99" s="1">
         <v>54.2</v>
       </c>
-      <c r="D99" s="1">
+      <c r="E99" s="1">
         <v>0.8</v>
       </c>
-      <c r="E99" s="1">
+      <c r="F99" s="1">
         <v>5.3</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B100" s="1">
+      <c r="B100" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C100" s="1">
         <v>32</v>
       </c>
-      <c r="C100" s="1">
+      <c r="D100" s="1">
         <v>38</v>
       </c>
-      <c r="D100" s="1">
+      <c r="E100" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E100" s="1">
+      <c r="F100" s="1">
         <v>6.8</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B101" s="1">
+      <c r="B101" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C101" s="1">
         <v>64</v>
       </c>
-      <c r="C101" s="1">
+      <c r="D101" s="1">
         <v>18.600000000000001</v>
       </c>
-      <c r="D101" s="1">
+      <c r="E101" s="1">
         <v>1.2</v>
       </c>
-      <c r="E101" s="1">
+      <c r="F101" s="1">
         <v>5.6</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B102" s="1">
+      <c r="B102" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C102" s="1">
         <v>80</v>
       </c>
-      <c r="C102" s="1">
+      <c r="D102" s="1">
         <v>13.6</v>
       </c>
-      <c r="D102" s="1">
+      <c r="E102" s="1">
         <v>1</v>
       </c>
-      <c r="E102" s="1">
+      <c r="F102" s="1">
         <v>4.2</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B103" s="1">
+      <c r="B103" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C103" s="1">
         <v>100</v>
       </c>
-      <c r="C103" s="1">
+      <c r="D103" s="1">
         <v>9.6</v>
       </c>
-      <c r="D103" s="1">
+      <c r="E103" s="1">
         <v>0.6</v>
       </c>
-      <c r="E103" s="1">
+      <c r="F103" s="1">
         <v>1.8</v>
       </c>
     </row>

</xml_diff>